<commit_message>
Content: 국문영문글정리 사용자 수정 반영 — 투자정보 세 장 히어로 문장 교체, 영문 이름(Smart Factory · Secondary Battery Activation/Materials · Automation System · Compound GaN Semiconductors · About · Company Intro · Reporting Center)을 같은 국문의 다른 줄 · 파생 문구에도 맞춤, 사전 다시 생성
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-export/국문영문글정리.xlsx
+++ b/content-export/국문영문글정리.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="9" activeTab="19" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" state="visible" r:id="rId1"/>
@@ -61,7 +61,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="맑은 고딕"/>
       <family val="2"/>
@@ -120,10 +120,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -152,22 +163,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F8"/>
+        <fgColor rgb="FFF4F6F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF6D6"/>
+        <fgColor rgb="FFFFF6D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F1FB"/>
+        <fgColor rgb="FFE8F1FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF9D9DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
       </patternFill>
     </fill>
   </fills>
@@ -196,23 +212,27 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D0D5DB"/>
+        <color rgb="FFD0D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00D0D5DB"/>
+        <color rgb="FFD0D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00D0D5DB"/>
+        <color rgb="FFD0D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D0D5DB"/>
+        <color rgb="FFD0D5DB"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -259,9 +279,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="강조색5" xfId="1" builtinId="45"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -922,7 +946,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="B49" s="2" t="inlineStr">
         <is>
           <t>페이지 영문 보기(KOR/ENG 단추)에 쓰는 글 중 다른 시트에 없는 것 — 메뉴 · 단추 · 사진 설명(대체 글) 등입니다. 엑셀이 이 글을 갖게 하려고 따로 모았습니다.</t>
@@ -1218,7 +1242,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
@@ -1260,7 +1284,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="16" t="n">
         <v>7</v>
       </c>
@@ -1478,7 +1502,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
@@ -1520,7 +1544,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="16" t="n">
         <v>13</v>
       </c>
@@ -1562,7 +1586,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="16" t="n">
         <v>14</v>
       </c>
@@ -1604,7 +1628,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="16" t="n">
         <v>15</v>
       </c>
@@ -1646,7 +1670,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="16" t="n">
         <v>16</v>
       </c>
@@ -1688,7 +1712,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="16" t="n">
         <v>17</v>
       </c>
@@ -2029,8 +2053,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="n">
+    <row r="3" ht="27" customHeight="1">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -2508,7 +2532,7 @@
       </c>
     </row>
     <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -2529,12 +2553,15 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>자연이 숨 쉬게 하는 기술력으로
-더불어 사는 세상을 만들어 갑니다.</t>
+          <t>A-PRO의 미래 가치와 투명한 기업 정보를 공유합니다.</t>
         </is>
       </c>
       <c r="G3" s="7" t="n"/>
-      <c r="H3" s="8" t="n"/>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>We share A-PRO's future value and transparent corporate information.</t>
+        </is>
+      </c>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="9" t="inlineStr">
         <is>
@@ -9576,8 +9603,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="n">
+    <row r="3" ht="27" customHeight="1">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -9598,13 +9625,13 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>투명하고 정확한 기업 정보를 적시에 공개합니다.</t>
+          <t>에이프로의 기업가치와 투자 정보를 투명하게 공개합니다.</t>
         </is>
       </c>
       <c r="G3" s="7" t="n"/>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>We disclose transparent and accurate corporate information in a timely manner.</t>
+          <t>We transparently disclose A-PRO's corporate value and investment information.</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -9618,7 +9645,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="27" customHeight="1">
       <c r="A4" s="16" t="n">
         <v>3</v>
       </c>
@@ -9778,7 +9805,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="16" t="n">
         <v>7</v>
       </c>
@@ -9888,7 +9915,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
@@ -14148,7 +14175,7 @@
       </c>
     </row>
     <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -14169,13 +14196,13 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>A-PRO의 미래 가치와 투명한 기업 정보를 공유합니다.</t>
+          <t>실시간 주가 정보와 시장 현황을 확인하실 수 있습니다.</t>
         </is>
       </c>
       <c r="G3" s="7" t="n"/>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>We share A-PRO's future value and transparent corporate information.</t>
+          <t>You can check real-time stock price and market status.</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -14362,7 +14389,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="16" t="n">
         <v>7</v>
       </c>
@@ -14446,7 +14473,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="16" t="n">
         <v>9</v>
       </c>
@@ -14488,7 +14515,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
@@ -14530,7 +14557,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="16" t="n">
         <v>11</v>
       </c>
@@ -14572,7 +14599,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
@@ -14614,7 +14641,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="16" t="n">
         <v>13</v>
       </c>
@@ -14656,7 +14683,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="16" t="n">
         <v>14</v>
       </c>
@@ -14970,7 +14997,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="16" t="n">
         <v>22</v>
       </c>
@@ -15012,7 +15039,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="16" t="n">
         <v>23</v>
       </c>
@@ -15054,7 +15081,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="16" t="n">
         <v>24</v>
       </c>
@@ -15096,7 +15123,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="16" t="n">
         <v>25</v>
       </c>
@@ -15138,7 +15165,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="16" t="n">
         <v>26</v>
       </c>
@@ -15222,7 +15249,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="16" t="n">
         <v>28</v>
       </c>
@@ -25283,7 +25310,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27" customHeight="1">
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
@@ -25541,7 +25568,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
@@ -25625,7 +25652,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
@@ -25709,7 +25736,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
@@ -25879,7 +25906,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="16" t="n">
         <v>16</v>
       </c>
@@ -25963,7 +25990,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="16" t="n">
         <v>18</v>
       </c>
@@ -26047,7 +26074,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="16" t="n">
         <v>20</v>
       </c>
@@ -26089,7 +26116,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="16" t="n">
         <v>21</v>
       </c>
@@ -27520,7 +27547,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27" customHeight="1">
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
@@ -27692,7 +27719,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
@@ -27776,7 +27803,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
@@ -27860,7 +27887,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
@@ -27944,7 +27971,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
@@ -29974,7 +30001,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="27" customHeight="1">
       <c r="A70" s="16" t="n">
         <v>69</v>
       </c>
@@ -30016,7 +30043,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="27" customHeight="1">
       <c r="A71" s="16" t="n">
         <v>70</v>
       </c>
@@ -30058,7 +30085,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="27" customHeight="1">
       <c r="A72" s="16" t="n">
         <v>71</v>
       </c>
@@ -30100,7 +30127,7 @@
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="27" customHeight="1">
       <c r="A73" s="16" t="n">
         <v>72</v>
       </c>
@@ -30142,7 +30169,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="27" customHeight="1">
       <c r="A74" s="16" t="n">
         <v>73</v>
       </c>
@@ -30184,7 +30211,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="27" customHeight="1">
       <c r="A75" s="16" t="n">
         <v>74</v>
       </c>
@@ -30226,7 +30253,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="27" customHeight="1">
       <c r="A76" s="16" t="n">
         <v>75</v>
       </c>
@@ -30310,7 +30337,7 @@
         </is>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="27" customHeight="1">
       <c r="A78" s="16" t="n">
         <v>77</v>
       </c>
@@ -32283,7 +32310,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27" customHeight="1">
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
@@ -33049,7 +33076,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="16" t="n">
         <v>21</v>
       </c>
@@ -36023,7 +36050,7 @@
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="27" customHeight="1">
       <c r="A93" s="16" t="n">
         <v>92</v>
       </c>
@@ -38866,7 +38893,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="27" customHeight="1">
       <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
@@ -38894,7 +38921,7 @@
       <c r="G2" s="7" t="n"/>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Reporting Channels</t>
+          <t>Reporting Center</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -38908,7 +38935,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27" customHeight="1">
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
@@ -39684,7 +39711,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="16" t="n">
         <v>20</v>
       </c>
@@ -39761,7 +39788,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="16" t="n">
         <v>22</v>
       </c>
@@ -39803,7 +39830,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="16" t="n">
         <v>23</v>
       </c>
@@ -39922,7 +39949,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="16" t="n">
         <v>26</v>
       </c>
@@ -39964,7 +39991,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="16" t="n">
         <v>27</v>
       </c>
@@ -40006,7 +40033,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="16" t="n">
         <v>28</v>
       </c>
@@ -40048,7 +40075,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="27" customHeight="1">
       <c r="A30" s="16" t="n">
         <v>29</v>
       </c>
@@ -40090,7 +40117,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="27" customHeight="1">
       <c r="A31" s="16" t="n">
         <v>30</v>
       </c>
@@ -40132,7 +40159,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="27" customHeight="1">
       <c r="A32" s="16" t="n">
         <v>31</v>
       </c>
@@ -40174,7 +40201,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="27" customHeight="1">
       <c r="A33" s="16" t="n">
         <v>32</v>
       </c>
@@ -40300,7 +40327,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="27" customHeight="1">
       <c r="A36" s="16" t="n">
         <v>35</v>
       </c>
@@ -40486,7 +40513,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="16" t="n">
         <v>40</v>
       </c>
@@ -40802,7 +40829,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="A49" s="16" t="n">
         <v>48</v>
       </c>
@@ -41039,7 +41066,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="27" customHeight="1">
       <c r="A4" s="16" t="n">
         <v>3</v>
       </c>
@@ -41081,8 +41108,8 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="16" t="n">
+    <row r="5" ht="27" customHeight="1">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -41124,7 +41151,7 @@
       </c>
     </row>
     <row r="6" ht="121.5" customHeight="1">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -41151,7 +41178,7 @@
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Smart Manufacturing</t>
+          <t>Smart Factory</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -41171,7 +41198,7 @@
       </c>
     </row>
     <row r="7" ht="121.5" customHeight="1">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -41218,7 +41245,7 @@
       </c>
     </row>
     <row r="8" ht="121.5" customHeight="1">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="18" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -41265,7 +41292,7 @@
       </c>
     </row>
     <row r="9" ht="135" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="18" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -41292,7 +41319,7 @@
       <c r="G9" s="7" t="n"/>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Compound Power Semiconductors</t>
+          <t>Compound GaN Semiconductors</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -41418,7 +41445,12 @@
         </is>
       </c>
       <c r="G12" s="7" t="n"/>
-      <c r="H12" s="8" t="n"/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>We develop and manufacture core equipment for the secondary battery activation process using our proprietary technologies.
+A-PRO takes full ownership of the final process that determines cell performance and quality.</t>
+        </is>
+      </c>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="9" t="inlineStr">
         <is>
@@ -41427,7 +41459,7 @@
       </c>
     </row>
     <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="18" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -41454,7 +41486,7 @@
       <c r="G13" s="7" t="n"/>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Battery Formation</t>
+          <t>Secondary Battery Activation</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -41512,7 +41544,7 @@
       </c>
     </row>
     <row r="15" ht="54" customHeight="1">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="18" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -41539,7 +41571,7 @@
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Automation Systems</t>
+          <t>Automation System</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -41582,7 +41614,7 @@
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Battery Materials</t>
+          <t>Secondary Battery Materials</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -42801,7 +42833,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="27" customHeight="1">
       <c r="A48" s="16" t="n">
         <v>47</v>
       </c>
@@ -43009,7 +43041,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27" customHeight="1">
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
@@ -43740,16 +43772,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J126"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="54" customWidth="1" min="7" max="7"/>
-    <col width="54" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="6" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
@@ -43806,7 +43836,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="27" customHeight="1">
       <c r="A2" s="17" t="n">
         <v>1</v>
       </c>
@@ -43834,7 +43864,7 @@
       <c r="G2" s="13" t="n"/>
       <c r="H2" s="14" t="inlineStr">
         <is>
-          <t>Compound Power Semiconductors</t>
+          <t>Compound GaN Semiconductors</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
@@ -43848,7 +43878,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="27" customHeight="1">
       <c r="A3" s="17" t="n">
         <v>2</v>
       </c>
@@ -43890,7 +43920,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="27" customHeight="1">
       <c r="A4" s="17" t="n">
         <v>3</v>
       </c>
@@ -43918,7 +43948,7 @@
       <c r="G4" s="13" t="n"/>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>About</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
@@ -43932,7 +43962,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="27" customHeight="1">
       <c r="A5" s="17" t="n">
         <v>4</v>
       </c>
@@ -43974,7 +44004,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="27" customHeight="1">
       <c r="A6" s="17" t="n">
         <v>5</v>
       </c>
@@ -44016,7 +44046,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="17" t="n">
         <v>6</v>
       </c>
@@ -44058,7 +44088,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="17" t="n">
         <v>7</v>
       </c>
@@ -44100,7 +44130,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="17" t="n">
         <v>8</v>
       </c>
@@ -44142,7 +44172,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="17" t="n">
         <v>9</v>
       </c>
@@ -44184,7 +44214,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="17" t="n">
         <v>10</v>
       </c>
@@ -44226,7 +44256,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="17" t="n">
         <v>11</v>
       </c>
@@ -44268,7 +44298,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="17" t="n">
         <v>12</v>
       </c>
@@ -44310,7 +44340,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="17" t="n">
         <v>13</v>
       </c>
@@ -44352,7 +44382,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="17" t="n">
         <v>14</v>
       </c>
@@ -44394,7 +44424,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="17" t="n">
         <v>15</v>
       </c>
@@ -44436,7 +44466,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="17" t="n">
         <v>16</v>
       </c>
@@ -44478,7 +44508,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="17" t="n">
         <v>17</v>
       </c>
@@ -44520,7 +44550,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="17" t="n">
         <v>18</v>
       </c>
@@ -44562,7 +44592,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="27" customHeight="1">
       <c r="A20" s="17" t="n">
         <v>19</v>
       </c>
@@ -44604,7 +44634,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="17" t="n">
         <v>20</v>
       </c>
@@ -44646,7 +44676,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="17" t="n">
         <v>21</v>
       </c>
@@ -44688,7 +44718,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="17" t="n">
         <v>22</v>
       </c>
@@ -44730,7 +44760,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="17" t="n">
         <v>23</v>
       </c>
@@ -44772,7 +44802,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="17" t="n">
         <v>24</v>
       </c>
@@ -44814,7 +44844,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="17" t="n">
         <v>25</v>
       </c>
@@ -44856,7 +44886,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="17" t="n">
         <v>26</v>
       </c>
@@ -44898,7 +44928,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="17" t="n">
         <v>27</v>
       </c>
@@ -44940,7 +44970,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="17" t="n">
         <v>28</v>
       </c>
@@ -44982,7 +45012,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="27" customHeight="1">
       <c r="A30" s="17" t="n">
         <v>29</v>
       </c>
@@ -45024,7 +45054,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="27" customHeight="1">
       <c r="A31" s="17" t="n">
         <v>30</v>
       </c>
@@ -45066,7 +45096,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="27" customHeight="1">
       <c r="A32" s="17" t="n">
         <v>31</v>
       </c>
@@ -45108,7 +45138,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="27" customHeight="1">
       <c r="A33" s="17" t="n">
         <v>32</v>
       </c>
@@ -45150,7 +45180,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="27" customHeight="1">
       <c r="A34" s="17" t="n">
         <v>33</v>
       </c>
@@ -45192,7 +45222,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="17" t="n">
         <v>34</v>
       </c>
@@ -45220,7 +45250,7 @@
       <c r="G35" s="13" t="n"/>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Smart Manufacturing categories</t>
+          <t>Smart Factory categories</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
@@ -45234,7 +45264,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="27" customHeight="1">
       <c r="A36" s="17" t="n">
         <v>35</v>
       </c>
@@ -45276,7 +45306,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="27" customHeight="1">
       <c r="A37" s="17" t="n">
         <v>36</v>
       </c>
@@ -45318,7 +45348,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="17" t="n">
         <v>37</v>
       </c>
@@ -45360,7 +45390,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="27" customHeight="1">
       <c r="A39" s="17" t="n">
         <v>38</v>
       </c>
@@ -45402,7 +45432,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="17" t="n">
         <v>39</v>
       </c>
@@ -45444,7 +45474,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="17" t="n">
         <v>40</v>
       </c>
@@ -45486,7 +45516,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="17" t="n">
         <v>41</v>
       </c>
@@ -45528,7 +45558,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="17" t="n">
         <v>42</v>
       </c>
@@ -45570,7 +45600,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="27" customHeight="1">
       <c r="A44" s="17" t="n">
         <v>43</v>
       </c>
@@ -45612,7 +45642,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="17" t="n">
         <v>44</v>
       </c>
@@ -45640,7 +45670,7 @@
       <c r="G45" s="13" t="n"/>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>Compound Power Semiconductors overview</t>
+          <t>Compound GaN Semiconductors overview</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
@@ -45654,7 +45684,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="27" customHeight="1">
       <c r="A46" s="17" t="n">
         <v>45</v>
       </c>
@@ -45698,7 +45728,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="27" customHeight="1">
       <c r="A47" s="17" t="n">
         <v>46</v>
       </c>
@@ -45740,7 +45770,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="27" customHeight="1">
       <c r="A48" s="17" t="n">
         <v>47</v>
       </c>
@@ -45768,7 +45798,7 @@
       <c r="G48" s="13" t="n"/>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>Smart Manufacturing overview</t>
+          <t>Smart Factory overview</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
@@ -45782,7 +45812,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="A49" s="17" t="n">
         <v>48</v>
       </c>
@@ -45824,7 +45854,7 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="27" customHeight="1">
       <c r="A50" s="17" t="n">
         <v>49</v>
       </c>
@@ -45866,7 +45896,7 @@
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="54" customHeight="1">
       <c r="A51" s="17" t="n">
         <v>50</v>
       </c>
@@ -45908,7 +45938,7 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="27" customHeight="1">
       <c r="A52" s="17" t="n">
         <v>51</v>
       </c>
@@ -45950,7 +45980,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="27" customHeight="1">
       <c r="A53" s="17" t="n">
         <v>52</v>
       </c>
@@ -45992,7 +46022,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="27" customHeight="1">
       <c r="A54" s="17" t="n">
         <v>53</v>
       </c>
@@ -46034,7 +46064,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="27" customHeight="1">
       <c r="A55" s="17" t="n">
         <v>54</v>
       </c>
@@ -46076,7 +46106,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="27" customHeight="1">
       <c r="A56" s="17" t="n">
         <v>55</v>
       </c>
@@ -46118,7 +46148,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="27" customHeight="1">
       <c r="A57" s="17" t="n">
         <v>56</v>
       </c>
@@ -46160,7 +46190,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="27" customHeight="1">
       <c r="A58" s="17" t="n">
         <v>57</v>
       </c>
@@ -46202,7 +46232,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="27" customHeight="1">
       <c r="A59" s="17" t="n">
         <v>58</v>
       </c>
@@ -46244,7 +46274,7 @@
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="40.5" customHeight="1">
       <c r="A60" s="17" t="n">
         <v>59</v>
       </c>
@@ -46286,7 +46316,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="27" customHeight="1">
       <c r="A61" s="17" t="n">
         <v>60</v>
       </c>
@@ -46328,7 +46358,7 @@
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="27" customHeight="1">
       <c r="A62" s="17" t="n">
         <v>61</v>
       </c>
@@ -46370,7 +46400,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="27" customHeight="1">
       <c r="A63" s="17" t="n">
         <v>62</v>
       </c>
@@ -46412,7 +46442,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="27" customHeight="1">
       <c r="A64" s="17" t="n">
         <v>63</v>
       </c>
@@ -46454,7 +46484,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="27" customHeight="1">
       <c r="A65" s="17" t="n">
         <v>64</v>
       </c>
@@ -46496,7 +46526,7 @@
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="27" customHeight="1">
       <c r="A66" s="17" t="n">
         <v>65</v>
       </c>
@@ -46538,7 +46568,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="27" customHeight="1">
       <c r="A67" s="17" t="n">
         <v>66</v>
       </c>
@@ -46580,7 +46610,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="27" customHeight="1">
       <c r="A68" s="17" t="n">
         <v>67</v>
       </c>
@@ -46622,7 +46652,7 @@
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="27" customHeight="1">
       <c r="A69" s="17" t="n">
         <v>68</v>
       </c>
@@ -46664,7 +46694,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="27" customHeight="1">
       <c r="A70" s="17" t="n">
         <v>69</v>
       </c>
@@ -46706,7 +46736,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="27" customHeight="1">
       <c r="A71" s="17" t="n">
         <v>70</v>
       </c>
@@ -46748,7 +46778,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="54" customHeight="1">
       <c r="A72" s="17" t="n">
         <v>71</v>
       </c>
@@ -46790,7 +46820,7 @@
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="27" customHeight="1">
       <c r="A73" s="17" t="n">
         <v>72</v>
       </c>
@@ -46832,7 +46862,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="27" customHeight="1">
       <c r="A74" s="17" t="n">
         <v>73</v>
       </c>
@@ -46874,7 +46904,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="27" customHeight="1">
       <c r="A75" s="17" t="n">
         <v>74</v>
       </c>
@@ -46916,7 +46946,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="27" customHeight="1">
       <c r="A76" s="17" t="n">
         <v>75</v>
       </c>
@@ -46958,7 +46988,7 @@
         </is>
       </c>
     </row>
-    <row r="77">
+    <row r="77" ht="27" customHeight="1">
       <c r="A77" s="17" t="n">
         <v>76</v>
       </c>
@@ -47000,7 +47030,7 @@
         </is>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="27" customHeight="1">
       <c r="A78" s="17" t="n">
         <v>77</v>
       </c>
@@ -47042,7 +47072,7 @@
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="27" customHeight="1">
       <c r="A79" s="17" t="n">
         <v>78</v>
       </c>
@@ -47084,7 +47114,7 @@
         </is>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="27" customHeight="1">
       <c r="A80" s="17" t="n">
         <v>79</v>
       </c>
@@ -47126,7 +47156,7 @@
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="27" customHeight="1">
       <c r="A81" s="17" t="n">
         <v>80</v>
       </c>
@@ -47170,7 +47200,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="27" customHeight="1">
       <c r="A82" s="17" t="n">
         <v>81</v>
       </c>
@@ -47212,7 +47242,7 @@
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="27" customHeight="1">
       <c r="A83" s="17" t="n">
         <v>82</v>
       </c>
@@ -47254,7 +47284,7 @@
         </is>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="27" customHeight="1">
       <c r="A84" s="17" t="n">
         <v>83</v>
       </c>
@@ -47296,7 +47326,7 @@
         </is>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="27" customHeight="1">
       <c r="A85" s="17" t="n">
         <v>84</v>
       </c>
@@ -47338,7 +47368,7 @@
         </is>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="27" customHeight="1">
       <c r="A86" s="17" t="n">
         <v>85</v>
       </c>
@@ -47380,7 +47410,7 @@
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="27" customHeight="1">
       <c r="A87" s="17" t="n">
         <v>86</v>
       </c>
@@ -47422,7 +47452,7 @@
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="27" customHeight="1">
       <c r="A88" s="17" t="n">
         <v>87</v>
       </c>
@@ -47464,7 +47494,7 @@
         </is>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="27" customHeight="1">
       <c r="A89" s="17" t="n">
         <v>88</v>
       </c>
@@ -47506,7 +47536,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="27" customHeight="1">
       <c r="A90" s="17" t="n">
         <v>89</v>
       </c>
@@ -47548,7 +47578,7 @@
         </is>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="27" customHeight="1">
       <c r="A91" s="17" t="n">
         <v>90</v>
       </c>
@@ -47590,7 +47620,7 @@
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="27" customHeight="1">
       <c r="A92" s="17" t="n">
         <v>91</v>
       </c>
@@ -47632,7 +47662,7 @@
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="27" customHeight="1">
       <c r="A93" s="17" t="n">
         <v>92</v>
       </c>
@@ -47660,7 +47690,7 @@
       <c r="G93" s="13" t="n"/>
       <c r="H93" s="14" t="inlineStr">
         <is>
-          <t>Expand Compound Power Semiconductors</t>
+          <t>Expand Compound GaN Semiconductors</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
@@ -47674,7 +47704,7 @@
         </is>
       </c>
     </row>
-    <row r="94">
+    <row r="94" ht="27" customHeight="1">
       <c r="A94" s="17" t="n">
         <v>93</v>
       </c>
@@ -47702,7 +47732,7 @@
       <c r="G94" s="13" t="n"/>
       <c r="H94" s="14" t="inlineStr">
         <is>
-          <t>Expand Smart Manufacturing</t>
+          <t>Expand Smart Factory</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
@@ -47716,7 +47746,7 @@
         </is>
       </c>
     </row>
-    <row r="95">
+    <row r="95" ht="27" customHeight="1">
       <c r="A95" s="17" t="n">
         <v>94</v>
       </c>
@@ -47758,7 +47788,7 @@
         </is>
       </c>
     </row>
-    <row r="96">
+    <row r="96" ht="27" customHeight="1">
       <c r="A96" s="17" t="n">
         <v>95</v>
       </c>
@@ -47800,7 +47830,7 @@
         </is>
       </c>
     </row>
-    <row r="97">
+    <row r="97" ht="67.5" customHeight="1">
       <c r="A97" s="17" t="n">
         <v>96</v>
       </c>
@@ -47842,7 +47872,7 @@
         </is>
       </c>
     </row>
-    <row r="98">
+    <row r="98" ht="27" customHeight="1">
       <c r="A98" s="17" t="n">
         <v>97</v>
       </c>
@@ -47884,7 +47914,7 @@
         </is>
       </c>
     </row>
-    <row r="99">
+    <row r="99" ht="27" customHeight="1">
       <c r="A99" s="17" t="n">
         <v>98</v>
       </c>
@@ -47926,7 +47956,7 @@
         </is>
       </c>
     </row>
-    <row r="100">
+    <row r="100" ht="27" customHeight="1">
       <c r="A100" s="17" t="n">
         <v>99</v>
       </c>
@@ -47968,7 +47998,7 @@
         </is>
       </c>
     </row>
-    <row r="101">
+    <row r="101" ht="27" customHeight="1">
       <c r="A101" s="17" t="n">
         <v>100</v>
       </c>
@@ -48010,7 +48040,7 @@
         </is>
       </c>
     </row>
-    <row r="102">
+    <row r="102" ht="27" customHeight="1">
       <c r="A102" s="17" t="n">
         <v>101</v>
       </c>
@@ -48052,7 +48082,7 @@
         </is>
       </c>
     </row>
-    <row r="103">
+    <row r="103" ht="27" customHeight="1">
       <c r="A103" s="17" t="n">
         <v>102</v>
       </c>
@@ -48094,7 +48124,7 @@
         </is>
       </c>
     </row>
-    <row r="104">
+    <row r="104" ht="27" customHeight="1">
       <c r="A104" s="17" t="n">
         <v>103</v>
       </c>
@@ -48136,7 +48166,7 @@
         </is>
       </c>
     </row>
-    <row r="105">
+    <row r="105" ht="27" customHeight="1">
       <c r="A105" s="17" t="n">
         <v>104</v>
       </c>
@@ -48178,7 +48208,7 @@
         </is>
       </c>
     </row>
-    <row r="106">
+    <row r="106" ht="27" customHeight="1">
       <c r="A106" s="17" t="n">
         <v>105</v>
       </c>
@@ -48220,7 +48250,7 @@
         </is>
       </c>
     </row>
-    <row r="107">
+    <row r="107" ht="27" customHeight="1">
       <c r="A107" s="17" t="n">
         <v>106</v>
       </c>
@@ -48262,7 +48292,7 @@
         </is>
       </c>
     </row>
-    <row r="108">
+    <row r="108" ht="27" customHeight="1">
       <c r="A108" s="17" t="n">
         <v>107</v>
       </c>
@@ -48304,7 +48334,7 @@
         </is>
       </c>
     </row>
-    <row r="109">
+    <row r="109" ht="27" customHeight="1">
       <c r="A109" s="17" t="n">
         <v>108</v>
       </c>
@@ -48346,7 +48376,7 @@
         </is>
       </c>
     </row>
-    <row r="110">
+    <row r="110" ht="27" customHeight="1">
       <c r="A110" s="17" t="n">
         <v>109</v>
       </c>
@@ -48388,7 +48418,7 @@
         </is>
       </c>
     </row>
-    <row r="111">
+    <row r="111" ht="27" customHeight="1">
       <c r="A111" s="17" t="n">
         <v>110</v>
       </c>
@@ -48430,7 +48460,7 @@
         </is>
       </c>
     </row>
-    <row r="112">
+    <row r="112" ht="27" customHeight="1">
       <c r="A112" s="17" t="n">
         <v>111</v>
       </c>
@@ -48472,7 +48502,7 @@
         </is>
       </c>
     </row>
-    <row r="113">
+    <row r="113" ht="27" customHeight="1">
       <c r="A113" s="17" t="n">
         <v>112</v>
       </c>
@@ -48514,7 +48544,7 @@
         </is>
       </c>
     </row>
-    <row r="114">
+    <row r="114" ht="27" customHeight="1">
       <c r="A114" s="17" t="n">
         <v>113</v>
       </c>
@@ -48556,7 +48586,7 @@
         </is>
       </c>
     </row>
-    <row r="115">
+    <row r="115" ht="27" customHeight="1">
       <c r="A115" s="17" t="n">
         <v>114</v>
       </c>
@@ -48598,7 +48628,7 @@
         </is>
       </c>
     </row>
-    <row r="116">
+    <row r="116" ht="27" customHeight="1">
       <c r="A116" s="17" t="n">
         <v>115</v>
       </c>
@@ -48642,7 +48672,7 @@
         </is>
       </c>
     </row>
-    <row r="117">
+    <row r="117" ht="27" customHeight="1">
       <c r="A117" s="17" t="n">
         <v>116</v>
       </c>
@@ -48684,7 +48714,7 @@
         </is>
       </c>
     </row>
-    <row r="118">
+    <row r="118" ht="27" customHeight="1">
       <c r="A118" s="17" t="n">
         <v>117</v>
       </c>
@@ -48728,7 +48758,7 @@
         </is>
       </c>
     </row>
-    <row r="119">
+    <row r="119" ht="27" customHeight="1">
       <c r="A119" s="17" t="n">
         <v>118</v>
       </c>
@@ -48770,7 +48800,7 @@
         </is>
       </c>
     </row>
-    <row r="120">
+    <row r="120" ht="27" customHeight="1">
       <c r="A120" s="17" t="n">
         <v>119</v>
       </c>
@@ -48814,7 +48844,7 @@
         </is>
       </c>
     </row>
-    <row r="121">
+    <row r="121" ht="27" customHeight="1">
       <c r="A121" s="17" t="n">
         <v>120</v>
       </c>
@@ -48858,7 +48888,7 @@
         </is>
       </c>
     </row>
-    <row r="122">
+    <row r="122" ht="27" customHeight="1">
       <c r="A122" s="17" t="n">
         <v>121</v>
       </c>
@@ -48902,7 +48932,7 @@
         </is>
       </c>
     </row>
-    <row r="123">
+    <row r="123" ht="27" customHeight="1">
       <c r="A123" s="17" t="n">
         <v>122</v>
       </c>
@@ -48946,7 +48976,7 @@
         </is>
       </c>
     </row>
-    <row r="124">
+    <row r="124" ht="27" customHeight="1">
       <c r="A124" s="17" t="n">
         <v>123</v>
       </c>
@@ -48988,7 +49018,7 @@
         </is>
       </c>
     </row>
-    <row r="125">
+    <row r="125" ht="27" customHeight="1">
       <c r="A125" s="17" t="n">
         <v>124</v>
       </c>
@@ -49030,7 +49060,7 @@
         </is>
       </c>
     </row>
-    <row r="126">
+    <row r="126" ht="27" customHeight="1">
       <c r="A126" s="17" t="n">
         <v>125</v>
       </c>
@@ -49368,7 +49398,7 @@
       </c>
     </row>
     <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -49395,7 +49425,7 @@
       <c r="G3" s="7" t="n"/>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Smart Manufacturing</t>
+          <t>Smart Factory</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -49411,7 +49441,7 @@
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="18" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -49454,7 +49484,7 @@
       </c>
     </row>
     <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -49497,7 +49527,7 @@
       </c>
     </row>
     <row r="6" ht="40.5" customHeight="1">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -49524,7 +49554,7 @@
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Compound Power Semiconductors</t>
+          <t>Compound GaN Semiconductors</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -49540,7 +49570,7 @@
       </c>
     </row>
     <row r="7" ht="40.5" customHeight="1">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -49567,7 +49597,7 @@
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>About</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -49583,7 +49613,7 @@
       </c>
     </row>
     <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="18" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -49610,7 +49640,7 @@
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>About Us</t>
+          <t>Company Intro</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -50013,7 +50043,7 @@
       </c>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="18" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -50034,11 +50064,15 @@
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>지배구조</t>
+          <t>거버넌스</t>
         </is>
       </c>
       <c r="G18" s="7" t="n"/>
-      <c r="H18" s="8" t="n"/>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
           <t>GNB · 메가 메뉴 · 전체 메뉴의 하위 이름과 같은 글</t>
@@ -50051,7 +50085,7 @@
       </c>
     </row>
     <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="16" t="n">
+      <c r="A19" s="18" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -50078,7 +50112,7 @@
       <c r="G19" s="7" t="n"/>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>Reporting Channels</t>
+          <t>Reporting Center</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -50265,7 +50299,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="16" t="n">
         <v>23</v>
       </c>
@@ -50307,7 +50341,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="16" t="n">
         <v>24</v>
       </c>
@@ -50349,7 +50383,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="16" t="n">
         <v>25</v>
       </c>
@@ -50391,7 +50425,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="16" t="n">
         <v>26</v>
       </c>
@@ -50703,7 +50737,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="16" t="n">
         <v>34</v>
       </c>
@@ -53748,8 +53782,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="16" t="n">
+    <row r="2" ht="27" customHeight="1">
+      <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -53776,7 +53810,7 @@
       <c r="G2" s="7" t="n"/>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Smart Manufacturing</t>
+          <t>Smart Factory</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -53947,7 +53981,7 @@
       </c>
     </row>
     <row r="7" ht="27" customHeight="1">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -53974,7 +54008,7 @@
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Battery Formation</t>
+          <t>Secondary Battery Activation</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -54036,7 +54070,7 @@
       </c>
     </row>
     <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="18" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -54063,7 +54097,7 @@
       <c r="G9" s="7" t="n"/>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Automation Systems</t>
+          <t>Automation System</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -54107,7 +54141,7 @@
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Battery Materials</t>
+          <t>Secondary Battery Materials</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -55058,7 +55092,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="27" customHeight="1">
       <c r="A34" s="16" t="n">
         <v>33</v>
       </c>
@@ -55100,7 +55134,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="16" t="n">
         <v>34</v>
       </c>
@@ -55142,7 +55176,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="27" customHeight="1">
       <c r="A36" s="16" t="n">
         <v>35</v>
       </c>
@@ -55184,7 +55218,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="27" customHeight="1">
       <c r="A37" s="16" t="n">
         <v>36</v>
       </c>
@@ -55226,7 +55260,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="16" t="n">
         <v>37</v>
       </c>
@@ -55268,7 +55302,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="27" customHeight="1">
       <c r="A39" s="16" t="n">
         <v>38</v>
       </c>
@@ -55310,7 +55344,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="16" t="n">
         <v>39</v>
       </c>
@@ -55352,7 +55386,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="16" t="n">
         <v>40</v>
       </c>
@@ -55394,7 +55428,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="16" t="n">
         <v>41</v>
       </c>
@@ -55436,7 +55470,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="16" t="n">
         <v>42</v>
       </c>
@@ -55478,7 +55512,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="27" customHeight="1">
       <c r="A44" s="16" t="n">
         <v>43</v>
       </c>
@@ -55520,7 +55554,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="16" t="n">
         <v>44</v>
       </c>
@@ -55562,7 +55596,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="27" customHeight="1">
       <c r="A46" s="16" t="n">
         <v>45</v>
       </c>
@@ -55604,7 +55638,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="27" customHeight="1">
       <c r="A47" s="16" t="n">
         <v>46</v>
       </c>
@@ -55646,7 +55680,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="27" customHeight="1">
       <c r="A48" s="16" t="n">
         <v>47</v>
       </c>
@@ -55688,7 +55722,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="A49" s="16" t="n">
         <v>48</v>
       </c>
@@ -55840,7 +55874,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="27" customHeight="1">
       <c r="A53" s="16" t="n">
         <v>52</v>
       </c>
@@ -55916,7 +55950,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="27" customHeight="1">
       <c r="A55" s="16" t="n">
         <v>54</v>
       </c>
@@ -55992,7 +56026,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="27" customHeight="1">
       <c r="A57" s="16" t="n">
         <v>56</v>
       </c>
@@ -56106,7 +56140,7 @@
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="27" customHeight="1">
       <c r="A60" s="16" t="n">
         <v>59</v>
       </c>
@@ -56224,7 +56258,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="27" customHeight="1">
       <c r="A63" s="16" t="n">
         <v>62</v>
       </c>
@@ -56300,7 +56334,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="27" customHeight="1">
       <c r="A65" s="16" t="n">
         <v>64</v>
       </c>
@@ -57178,7 +57212,7 @@
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="27" customHeight="1">
       <c r="A88" s="16" t="n">
         <v>87</v>
       </c>
@@ -57220,7 +57254,7 @@
         </is>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="27" customHeight="1">
       <c r="A89" s="16" t="n">
         <v>88</v>
       </c>
@@ -57262,7 +57296,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="27" customHeight="1">
       <c r="A90" s="16" t="n">
         <v>89</v>
       </c>
@@ -57346,7 +57380,7 @@
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="27" customHeight="1">
       <c r="A92" s="16" t="n">
         <v>91</v>
       </c>
@@ -57388,7 +57422,7 @@
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="27" customHeight="1">
       <c r="A93" s="16" t="n">
         <v>92</v>
       </c>
@@ -57430,7 +57464,7 @@
         </is>
       </c>
     </row>
-    <row r="94">
+    <row r="94" ht="27" customHeight="1">
       <c r="A94" s="16" t="n">
         <v>93</v>
       </c>
@@ -57780,7 +57814,7 @@
         </is>
       </c>
     </row>
-    <row r="103">
+    <row r="103" ht="27" customHeight="1">
       <c r="A103" s="16" t="n">
         <v>102</v>
       </c>
@@ -57822,7 +57856,7 @@
         </is>
       </c>
     </row>
-    <row r="104">
+    <row r="104" ht="27" customHeight="1">
       <c r="A104" s="16" t="n">
         <v>103</v>
       </c>
@@ -57864,7 +57898,7 @@
         </is>
       </c>
     </row>
-    <row r="105">
+    <row r="105" ht="27" customHeight="1">
       <c r="A105" s="16" t="n">
         <v>104</v>
       </c>
@@ -57906,7 +57940,7 @@
         </is>
       </c>
     </row>
-    <row r="106">
+    <row r="106" ht="27" customHeight="1">
       <c r="A106" s="16" t="n">
         <v>105</v>
       </c>
@@ -57948,7 +57982,7 @@
         </is>
       </c>
     </row>
-    <row r="107">
+    <row r="107" ht="27" customHeight="1">
       <c r="A107" s="16" t="n">
         <v>106</v>
       </c>
@@ -57990,7 +58024,7 @@
         </is>
       </c>
     </row>
-    <row r="108">
+    <row r="108" ht="27" customHeight="1">
       <c r="A108" s="16" t="n">
         <v>107</v>
       </c>
@@ -58032,7 +58066,7 @@
         </is>
       </c>
     </row>
-    <row r="109">
+    <row r="109" ht="27" customHeight="1">
       <c r="A109" s="16" t="n">
         <v>108</v>
       </c>
@@ -58074,7 +58108,7 @@
         </is>
       </c>
     </row>
-    <row r="110">
+    <row r="110" ht="27" customHeight="1">
       <c r="A110" s="16" t="n">
         <v>109</v>
       </c>
@@ -58116,7 +58150,7 @@
         </is>
       </c>
     </row>
-    <row r="111">
+    <row r="111" ht="27" customHeight="1">
       <c r="A111" s="16" t="n">
         <v>110</v>
       </c>
@@ -58158,7 +58192,7 @@
         </is>
       </c>
     </row>
-    <row r="112">
+    <row r="112" ht="27" customHeight="1">
       <c r="A112" s="16" t="n">
         <v>111</v>
       </c>
@@ -58200,7 +58234,7 @@
         </is>
       </c>
     </row>
-    <row r="113">
+    <row r="113" ht="27" customHeight="1">
       <c r="A113" s="16" t="n">
         <v>112</v>
       </c>
@@ -58242,7 +58276,7 @@
         </is>
       </c>
     </row>
-    <row r="114">
+    <row r="114" ht="27" customHeight="1">
       <c r="A114" s="16" t="n">
         <v>113</v>
       </c>
@@ -58284,7 +58318,7 @@
         </is>
       </c>
     </row>
-    <row r="115">
+    <row r="115" ht="27" customHeight="1">
       <c r="A115" s="16" t="n">
         <v>114</v>
       </c>
@@ -58326,7 +58360,7 @@
         </is>
       </c>
     </row>
-    <row r="116">
+    <row r="116" ht="27" customHeight="1">
       <c r="A116" s="16" t="n">
         <v>115</v>
       </c>
@@ -58368,7 +58402,7 @@
         </is>
       </c>
     </row>
-    <row r="117">
+    <row r="117" ht="27" customHeight="1">
       <c r="A117" s="16" t="n">
         <v>116</v>
       </c>
@@ -58520,7 +58554,7 @@
         </is>
       </c>
     </row>
-    <row r="121">
+    <row r="121" ht="27" customHeight="1">
       <c r="A121" s="16" t="n">
         <v>120</v>
       </c>
@@ -58596,7 +58630,7 @@
         </is>
       </c>
     </row>
-    <row r="123">
+    <row r="123" ht="27" customHeight="1">
       <c r="A123" s="16" t="n">
         <v>122</v>
       </c>
@@ -58672,7 +58706,7 @@
         </is>
       </c>
     </row>
-    <row r="125">
+    <row r="125" ht="27" customHeight="1">
       <c r="A125" s="16" t="n">
         <v>124</v>
       </c>
@@ -58748,7 +58782,7 @@
         </is>
       </c>
     </row>
-    <row r="127">
+    <row r="127" ht="27" customHeight="1">
       <c r="A127" s="16" t="n">
         <v>126</v>
       </c>
@@ -58824,7 +58858,7 @@
         </is>
       </c>
     </row>
-    <row r="129">
+    <row r="129" ht="27" customHeight="1">
       <c r="A129" s="16" t="n">
         <v>128</v>
       </c>
@@ -59014,7 +59048,7 @@
         </is>
       </c>
     </row>
-    <row r="134">
+    <row r="134" ht="27" customHeight="1">
       <c r="A134" s="16" t="n">
         <v>133</v>
       </c>
@@ -59090,7 +59124,7 @@
         </is>
       </c>
     </row>
-    <row r="136">
+    <row r="136" ht="27" customHeight="1">
       <c r="A136" s="16" t="n">
         <v>135</v>
       </c>
@@ -59166,7 +59200,7 @@
         </is>
       </c>
     </row>
-    <row r="138">
+    <row r="138" ht="27" customHeight="1">
       <c r="A138" s="16" t="n">
         <v>137</v>
       </c>
@@ -59242,7 +59276,7 @@
         </is>
       </c>
     </row>
-    <row r="140">
+    <row r="140" ht="27" customHeight="1">
       <c r="A140" s="16" t="n">
         <v>139</v>
       </c>
@@ -59361,8 +59395,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="16" t="n">
+    <row r="2" ht="27" customHeight="1">
+      <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -60254,7 +60288,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="16" t="n">
         <v>23</v>
       </c>
@@ -60296,7 +60330,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="16" t="n">
         <v>24</v>
       </c>
@@ -60338,7 +60372,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="16" t="n">
         <v>25</v>
       </c>
@@ -60380,7 +60414,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="16" t="n">
         <v>26</v>
       </c>
@@ -60422,7 +60456,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="16" t="n">
         <v>27</v>
       </c>
@@ -60464,7 +60498,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="16" t="n">
         <v>28</v>
       </c>
@@ -62759,7 +62793,7 @@
         </is>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="27" customHeight="1">
       <c r="A91" s="16" t="n">
         <v>90</v>
       </c>
@@ -62801,7 +62835,7 @@
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="27" customHeight="1">
       <c r="A92" s="16" t="n">
         <v>91</v>
       </c>
@@ -63283,7 +63317,7 @@
         </is>
       </c>
     </row>
-    <row r="103">
+    <row r="103" ht="27" customHeight="1">
       <c r="A103" s="16" t="n">
         <v>102</v>
       </c>
@@ -63325,7 +63359,7 @@
         </is>
       </c>
     </row>
-    <row r="104">
+    <row r="104" ht="27" customHeight="1">
       <c r="A104" s="16" t="n">
         <v>103</v>
       </c>
@@ -63750,7 +63784,7 @@
         </is>
       </c>
     </row>
-    <row r="114">
+    <row r="114" ht="27" customHeight="1">
       <c r="A114" s="16" t="n">
         <v>113</v>
       </c>
@@ -64166,7 +64200,7 @@
         </is>
       </c>
     </row>
-    <row r="124">
+    <row r="124" ht="27" customHeight="1">
       <c r="A124" s="16" t="n">
         <v>123</v>
       </c>
@@ -64574,7 +64608,7 @@
         </is>
       </c>
     </row>
-    <row r="134">
+    <row r="134" ht="27" customHeight="1">
       <c r="A134" s="16" t="n">
         <v>133</v>
       </c>
@@ -64948,7 +64982,7 @@
         </is>
       </c>
     </row>
-    <row r="143">
+    <row r="143" ht="27" customHeight="1">
       <c r="A143" s="16" t="n">
         <v>142</v>
       </c>
@@ -65222,7 +65256,7 @@
         </is>
       </c>
     </row>
-    <row r="150">
+    <row r="150" ht="27" customHeight="1">
       <c r="A150" s="16" t="n">
         <v>149</v>
       </c>
@@ -65638,7 +65672,7 @@
         </is>
       </c>
     </row>
-    <row r="160">
+    <row r="160" ht="27" customHeight="1">
       <c r="A160" s="16" t="n">
         <v>159</v>
       </c>
@@ -66054,7 +66088,7 @@
         </is>
       </c>
     </row>
-    <row r="170">
+    <row r="170" ht="27" customHeight="1">
       <c r="A170" s="16" t="n">
         <v>169</v>
       </c>
@@ -66547,7 +66581,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="27" customHeight="1">
       <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
@@ -67306,7 +67340,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="16" t="n">
         <v>20</v>
       </c>
@@ -67390,7 +67424,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="16" t="n">
         <v>22</v>
       </c>
@@ -67432,7 +67466,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="16" t="n">
         <v>23</v>
       </c>
@@ -67474,7 +67508,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="16" t="n">
         <v>24</v>
       </c>
@@ -67516,7 +67550,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="16" t="n">
         <v>25</v>
       </c>
@@ -67600,7 +67634,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="16" t="n">
         <v>27</v>
       </c>
@@ -68477,7 +68511,7 @@
       <c r="G2" s="7" t="n"/>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Compound Power Semiconductors</t>
+          <t>Compound GaN Semiconductors</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -68918,7 +68952,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="16" t="n">
         <v>13</v>
       </c>
@@ -68960,7 +68994,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="16" t="n">
         <v>14</v>
       </c>
@@ -69002,7 +69036,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="16" t="n">
         <v>15</v>
       </c>
@@ -69410,7 +69444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -69475,7 +69509,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="27" customHeight="1">
       <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
@@ -69517,8 +69551,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="n">
+    <row r="3" ht="27" customHeight="1">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -69545,7 +69579,7 @@
       <c r="G3" s="7" t="n"/>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Smart Manufacturing</t>
+          <t>Smart Factory</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -69597,8 +69631,8 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="16" t="n">
+    <row r="5" ht="27" customHeight="1">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -69625,7 +69659,7 @@
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Battery Formation</t>
+          <t>Secondary Battery Activation</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -69677,7 +69711,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
@@ -69705,7 +69739,7 @@
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Automation Systems</t>
+          <t>Automation System</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -69719,7 +69753,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="16" t="n">
         <v>7</v>
       </c>
@@ -69747,7 +69781,7 @@
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Battery Materials</t>
+          <t>Secondary Battery Materials</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -69805,8 +69839,8 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="16" t="n">
+    <row r="10" ht="27" customHeight="1">
+      <c r="A10" s="18" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -69999,8 +70033,8 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="16" t="n">
+    <row r="15" ht="27" customHeight="1">
+      <c r="A15" s="18" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -70079,7 +70113,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="16" t="n">
         <v>16</v>
       </c>
@@ -70121,7 +70155,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="16" t="n">
         <v>17</v>
       </c>
@@ -70267,7 +70301,7 @@
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>Compound Power Semiconductors</t>
+          <t>Compound GaN Semiconductors</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -70434,48 +70468,6 @@
       <c r="J25" s="9" t="inlineStr">
         <is>
           <t>/html/body/section/div/a[4]/div[2]/span[3]/span[2]|text</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>본문</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>글</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>문구</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>데스크톱(1280px 이상) 기준으로 디자인된 시안입니다.</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>This draft is designed for desktop (1280px and wider).</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>영문 초벌 번역(Claude, 2026-10-08) — 검토 필요</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="inlineStr">
-        <is>
-          <t>/html/body/div[1]|text</t>
         </is>
       </c>
     </row>
@@ -70823,7 +70815,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
@@ -70943,7 +70935,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="16" t="n">
         <v>11</v>
       </c>
@@ -71063,7 +71055,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="16" t="n">
         <v>14</v>
       </c>

</xml_diff>